<commit_message>
Actualización Proyecto Aurelion 23-12-2025
Actualización Final Proyecto Tienda Aurelion.
</commit_message>
<xml_diff>
--- a/Carlos Padilla - Proyecto Aurelion/clientes.xlsx
+++ b/Carlos Padilla - Proyecto Aurelion/clientes.xlsx
@@ -1,17 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\capab\OneDrive\Escritorio\Certificación IA IBM\Clases Sincrónicas y Proyecto\Proyecto-Aurelion-IBM\Carlos Padilla - Proyecto Aurelion\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5C2267A-2FF4-4F32-89DF-784282EC336B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="clientes.csv" sheetId="1" r:id="rId4"/>
+    <sheet name="clientes.csv" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'clientes.csv'!$A$1:$F$101</definedName>
+  </definedNames>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="209">
   <si>
     <t>id_cliente</t>
   </si>
@@ -629,23 +641,33 @@
   </si>
   <si>
     <t>agustina.lopez@mail.com</t>
+  </si>
+  <si>
+    <t>Sexo</t>
+  </si>
+  <si>
+    <t>Femenino</t>
+  </si>
+  <si>
+    <t>Masculino</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -656,39 +678,44 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -878,17 +905,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F101"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -904,10 +934,13 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="F1" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>5</v>
@@ -919,12 +952,15 @@
         <v>7</v>
       </c>
       <c r="E2" s="2">
-        <v>44927.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>44927</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>8</v>
@@ -936,12 +972,15 @@
         <v>7</v>
       </c>
       <c r="E3" s="2">
-        <v>44928.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>44928</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>10</v>
@@ -953,12 +992,15 @@
         <v>12</v>
       </c>
       <c r="E4" s="2">
-        <v>44929.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>44929</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>13</v>
@@ -970,12 +1012,15 @@
         <v>7</v>
       </c>
       <c r="E5" s="2">
-        <v>44930.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>44930</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>15</v>
@@ -987,12 +1032,15 @@
         <v>17</v>
       </c>
       <c r="E6" s="2">
-        <v>44931.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>44931</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -1004,12 +1052,15 @@
         <v>20</v>
       </c>
       <c r="E7" s="2">
-        <v>44932.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>44932</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>21</v>
@@ -1021,12 +1072,15 @@
         <v>12</v>
       </c>
       <c r="E8" s="2">
-        <v>44933.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>44933</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>23</v>
@@ -1038,12 +1092,15 @@
         <v>7</v>
       </c>
       <c r="E9" s="2">
-        <v>44934.0</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>44934</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>25</v>
@@ -1055,12 +1112,15 @@
         <v>7</v>
       </c>
       <c r="E10" s="2">
-        <v>44935.0</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>44935</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>27</v>
@@ -1072,12 +1132,15 @@
         <v>17</v>
       </c>
       <c r="E11" s="2">
-        <v>44936.0</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>44936</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>29</v>
@@ -1089,12 +1152,15 @@
         <v>20</v>
       </c>
       <c r="E12" s="2">
-        <v>44937.0</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>44937</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>31</v>
@@ -1106,12 +1172,15 @@
         <v>33</v>
       </c>
       <c r="E13" s="2">
-        <v>44938.0</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>44938</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>13.0</v>
+        <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>34</v>
@@ -1123,12 +1192,15 @@
         <v>7</v>
       </c>
       <c r="E14" s="2">
-        <v>44939.0</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>44939</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>36</v>
@@ -1140,12 +1212,15 @@
         <v>7</v>
       </c>
       <c r="E15" s="2">
-        <v>44940.0</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>44940</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>38</v>
@@ -1157,12 +1232,15 @@
         <v>17</v>
       </c>
       <c r="E16" s="2">
-        <v>44941.0</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>44941</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>16.0</v>
+        <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>40</v>
@@ -1174,12 +1252,15 @@
         <v>12</v>
       </c>
       <c r="E17" s="2">
-        <v>44942.0</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>44942</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>42</v>
@@ -1191,12 +1272,15 @@
         <v>20</v>
       </c>
       <c r="E18" s="2">
-        <v>44943.0</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>44943</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>44</v>
@@ -1208,12 +1292,15 @@
         <v>7</v>
       </c>
       <c r="E19" s="2">
-        <v>44944.0</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>44944</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>46</v>
@@ -1225,12 +1312,15 @@
         <v>48</v>
       </c>
       <c r="E20" s="2">
-        <v>44945.0</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>44945</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>49</v>
@@ -1242,12 +1332,15 @@
         <v>12</v>
       </c>
       <c r="E21" s="2">
-        <v>44946.0</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>44946</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>51</v>
@@ -1259,12 +1352,15 @@
         <v>33</v>
       </c>
       <c r="E22" s="2">
-        <v>44947.0</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>44947</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>53</v>
@@ -1276,12 +1372,15 @@
         <v>33</v>
       </c>
       <c r="E23" s="2">
-        <v>44948.0</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>44948</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>23.0</v>
+        <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>55</v>
@@ -1293,12 +1392,15 @@
         <v>12</v>
       </c>
       <c r="E24" s="2">
-        <v>44949.0</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>44949</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>57</v>
@@ -1310,12 +1412,15 @@
         <v>20</v>
       </c>
       <c r="E25" s="2">
-        <v>44950.0</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>44950</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>59</v>
@@ -1327,12 +1432,15 @@
         <v>12</v>
       </c>
       <c r="E26" s="2">
-        <v>44951.0</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>44951</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>26.0</v>
+        <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>61</v>
@@ -1344,12 +1452,15 @@
         <v>33</v>
       </c>
       <c r="E27" s="2">
-        <v>44952.0</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>44952</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>27.0</v>
+        <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>63</v>
@@ -1361,12 +1472,15 @@
         <v>12</v>
       </c>
       <c r="E28" s="2">
-        <v>44953.0</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>44953</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>65</v>
@@ -1378,12 +1492,15 @@
         <v>17</v>
       </c>
       <c r="E29" s="2">
-        <v>44954.0</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>44954</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>29.0</v>
+        <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>67</v>
@@ -1395,12 +1512,15 @@
         <v>33</v>
       </c>
       <c r="E30" s="2">
-        <v>44955.0</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>44955</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>69</v>
@@ -1412,12 +1532,15 @@
         <v>33</v>
       </c>
       <c r="E31" s="2">
-        <v>44956.0</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>44956</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>31.0</v>
+        <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>71</v>
@@ -1429,12 +1552,15 @@
         <v>20</v>
       </c>
       <c r="E32" s="2">
-        <v>44957.0</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>44957</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>73</v>
@@ -1446,12 +1572,15 @@
         <v>48</v>
       </c>
       <c r="E33" s="2">
-        <v>44958.0</v>
-      </c>
-    </row>
-    <row r="34">
+        <v>44958</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>33.0</v>
+        <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>75</v>
@@ -1463,12 +1592,15 @@
         <v>12</v>
       </c>
       <c r="E34" s="2">
-        <v>44959.0</v>
-      </c>
-    </row>
-    <row r="35">
+        <v>44959</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>34.0</v>
+        <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>23</v>
@@ -1480,12 +1612,15 @@
         <v>20</v>
       </c>
       <c r="E35" s="2">
-        <v>44960.0</v>
-      </c>
-    </row>
-    <row r="36">
+        <v>44960</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>35.0</v>
+        <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>78</v>
@@ -1497,12 +1632,15 @@
         <v>48</v>
       </c>
       <c r="E36" s="2">
-        <v>44961.0</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>44961</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>36.0</v>
+        <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>80</v>
@@ -1514,12 +1652,15 @@
         <v>48</v>
       </c>
       <c r="E37" s="2">
-        <v>44962.0</v>
-      </c>
-    </row>
-    <row r="38">
+        <v>44962</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>37.0</v>
+        <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>82</v>
@@ -1531,12 +1672,15 @@
         <v>48</v>
       </c>
       <c r="E38" s="2">
-        <v>44963.0</v>
-      </c>
-    </row>
-    <row r="39">
+        <v>44963</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>38.0</v>
+        <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>84</v>
@@ -1548,12 +1692,15 @@
         <v>33</v>
       </c>
       <c r="E39" s="2">
-        <v>44964.0</v>
-      </c>
-    </row>
-    <row r="40">
+        <v>44964</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>39.0</v>
+        <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>86</v>
@@ -1565,12 +1712,15 @@
         <v>33</v>
       </c>
       <c r="E40" s="2">
-        <v>44965.0</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>44965</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>88</v>
@@ -1582,12 +1732,15 @@
         <v>12</v>
       </c>
       <c r="E41" s="2">
-        <v>44966.0</v>
-      </c>
-    </row>
-    <row r="42">
+        <v>44966</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>41.0</v>
+        <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>51</v>
@@ -1599,12 +1752,15 @@
         <v>33</v>
       </c>
       <c r="E42" s="2">
-        <v>44967.0</v>
-      </c>
-    </row>
-    <row r="43">
+        <v>44967</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>42.0</v>
+        <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>91</v>
@@ -1616,12 +1772,15 @@
         <v>33</v>
       </c>
       <c r="E43" s="2">
-        <v>44968.0</v>
-      </c>
-    </row>
-    <row r="44">
+        <v>44968</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>43.0</v>
+        <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>93</v>
@@ -1633,12 +1792,15 @@
         <v>48</v>
       </c>
       <c r="E44" s="2">
-        <v>44969.0</v>
-      </c>
-    </row>
-    <row r="45">
+        <v>44969</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>44.0</v>
+        <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>95</v>
@@ -1650,12 +1812,15 @@
         <v>7</v>
       </c>
       <c r="E45" s="2">
-        <v>44970.0</v>
-      </c>
-    </row>
-    <row r="46">
+        <v>44970</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>45.0</v>
+        <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>97</v>
@@ -1667,12 +1832,15 @@
         <v>12</v>
       </c>
       <c r="E46" s="2">
-        <v>44971.0</v>
-      </c>
-    </row>
-    <row r="47">
+        <v>44971</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>46.0</v>
+        <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>99</v>
@@ -1684,12 +1852,15 @@
         <v>33</v>
       </c>
       <c r="E47" s="2">
-        <v>44972.0</v>
-      </c>
-    </row>
-    <row r="48">
+        <v>44972</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>47.0</v>
+        <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>101</v>
@@ -1701,12 +1872,15 @@
         <v>33</v>
       </c>
       <c r="E48" s="2">
-        <v>44973.0</v>
-      </c>
-    </row>
-    <row r="49">
+        <v>44973</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>48.0</v>
+        <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>103</v>
@@ -1718,12 +1892,15 @@
         <v>17</v>
       </c>
       <c r="E49" s="2">
-        <v>44974.0</v>
-      </c>
-    </row>
-    <row r="50">
+        <v>44974</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>49.0</v>
+        <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>105</v>
@@ -1735,12 +1912,15 @@
         <v>12</v>
       </c>
       <c r="E50" s="2">
-        <v>44975.0</v>
-      </c>
-    </row>
-    <row r="51">
+        <v>44975</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>107</v>
@@ -1752,12 +1932,15 @@
         <v>7</v>
       </c>
       <c r="E51" s="2">
-        <v>44976.0</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>44976</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>51.0</v>
+        <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>109</v>
@@ -1769,12 +1952,15 @@
         <v>12</v>
       </c>
       <c r="E52" s="2">
-        <v>44977.0</v>
-      </c>
-    </row>
-    <row r="53">
+        <v>44977</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>52.0</v>
+        <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>111</v>
@@ -1786,12 +1972,15 @@
         <v>12</v>
       </c>
       <c r="E53" s="2">
-        <v>44978.0</v>
-      </c>
-    </row>
-    <row r="54">
+        <v>44978</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>53.0</v>
+        <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>113</v>
@@ -1803,12 +1992,15 @@
         <v>48</v>
       </c>
       <c r="E54" s="2">
-        <v>44979.0</v>
-      </c>
-    </row>
-    <row r="55">
+        <v>44979</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>54.0</v>
+        <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>115</v>
@@ -1820,12 +2012,15 @@
         <v>33</v>
       </c>
       <c r="E55" s="2">
-        <v>44980.0</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>44980</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>55.0</v>
+        <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>117</v>
@@ -1837,12 +2032,15 @@
         <v>48</v>
       </c>
       <c r="E56" s="2">
-        <v>44981.0</v>
-      </c>
-    </row>
-    <row r="57">
+        <v>44981</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>56.0</v>
+        <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>119</v>
@@ -1854,12 +2052,15 @@
         <v>12</v>
       </c>
       <c r="E57" s="2">
-        <v>44982.0</v>
-      </c>
-    </row>
-    <row r="58">
+        <v>44982</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>57.0</v>
+        <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>121</v>
@@ -1871,12 +2072,15 @@
         <v>12</v>
       </c>
       <c r="E58" s="2">
-        <v>44983.0</v>
-      </c>
-    </row>
-    <row r="59">
+        <v>44983</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>58.0</v>
+        <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>27</v>
@@ -1888,12 +2092,15 @@
         <v>12</v>
       </c>
       <c r="E59" s="2">
-        <v>44984.0</v>
-      </c>
-    </row>
-    <row r="60">
+        <v>44984</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>59.0</v>
+        <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>124</v>
@@ -1905,12 +2112,15 @@
         <v>20</v>
       </c>
       <c r="E60" s="2">
-        <v>44985.0</v>
-      </c>
-    </row>
-    <row r="61">
+        <v>44985</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>60.0</v>
+        <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>126</v>
@@ -1922,12 +2132,15 @@
         <v>33</v>
       </c>
       <c r="E61" s="2">
-        <v>44986.0</v>
-      </c>
-    </row>
-    <row r="62">
+        <v>44986</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>61.0</v>
+        <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>128</v>
@@ -1939,12 +2152,15 @@
         <v>12</v>
       </c>
       <c r="E62" s="2">
-        <v>44987.0</v>
-      </c>
-    </row>
-    <row r="63">
+        <v>44987</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>62.0</v>
+        <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>130</v>
@@ -1956,12 +2172,15 @@
         <v>7</v>
       </c>
       <c r="E63" s="2">
-        <v>44988.0</v>
-      </c>
-    </row>
-    <row r="64">
+        <v>44988</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>63.0</v>
+        <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>132</v>
@@ -1973,12 +2192,15 @@
         <v>17</v>
       </c>
       <c r="E64" s="2">
-        <v>44989.0</v>
-      </c>
-    </row>
-    <row r="65">
+        <v>44989</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>64.0</v>
+        <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>134</v>
@@ -1990,12 +2212,15 @@
         <v>20</v>
       </c>
       <c r="E65" s="2">
-        <v>44990.0</v>
-      </c>
-    </row>
-    <row r="66">
+        <v>44990</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>65.0</v>
+        <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>136</v>
@@ -2007,12 +2232,15 @@
         <v>33</v>
       </c>
       <c r="E66" s="2">
-        <v>44991.0</v>
-      </c>
-    </row>
-    <row r="67">
+        <v>44991</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>66.0</v>
+        <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>138</v>
@@ -2024,12 +2252,15 @@
         <v>20</v>
       </c>
       <c r="E67" s="2">
-        <v>44992.0</v>
-      </c>
-    </row>
-    <row r="68">
+        <v>44992</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>67.0</v>
+        <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>140</v>
@@ -2041,12 +2272,15 @@
         <v>33</v>
       </c>
       <c r="E68" s="2">
-        <v>44993.0</v>
-      </c>
-    </row>
-    <row r="69">
+        <v>44993</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>68.0</v>
+        <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>142</v>
@@ -2058,12 +2292,15 @@
         <v>20</v>
       </c>
       <c r="E69" s="2">
-        <v>44994.0</v>
-      </c>
-    </row>
-    <row r="70">
+        <v>44994</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>69.0</v>
+        <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>144</v>
@@ -2075,12 +2312,15 @@
         <v>12</v>
       </c>
       <c r="E70" s="2">
-        <v>44995.0</v>
-      </c>
-    </row>
-    <row r="71">
+        <v>44995</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>70.0</v>
+        <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>146</v>
@@ -2092,12 +2332,15 @@
         <v>7</v>
       </c>
       <c r="E71" s="2">
-        <v>44996.0</v>
-      </c>
-    </row>
-    <row r="72">
+        <v>44996</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>71.0</v>
+        <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>148</v>
@@ -2109,12 +2352,15 @@
         <v>20</v>
       </c>
       <c r="E72" s="2">
-        <v>44997.0</v>
-      </c>
-    </row>
-    <row r="73">
+        <v>44997</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>72.0</v>
+        <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>150</v>
@@ -2126,12 +2372,15 @@
         <v>17</v>
       </c>
       <c r="E73" s="2">
-        <v>44998.0</v>
-      </c>
-    </row>
-    <row r="74">
+        <v>44998</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>73.0</v>
+        <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>152</v>
@@ -2143,12 +2392,15 @@
         <v>33</v>
       </c>
       <c r="E74" s="2">
-        <v>44999.0</v>
-      </c>
-    </row>
-    <row r="75">
+        <v>44999</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>74.0</v>
+        <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>154</v>
@@ -2160,12 +2412,15 @@
         <v>7</v>
       </c>
       <c r="E75" s="2">
-        <v>45000.0</v>
-      </c>
-    </row>
-    <row r="76">
+        <v>45000</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>75.0</v>
+        <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>156</v>
@@ -2177,12 +2432,15 @@
         <v>12</v>
       </c>
       <c r="E76" s="2">
-        <v>45001.0</v>
-      </c>
-    </row>
-    <row r="77">
+        <v>45001</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>76.0</v>
+        <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>158</v>
@@ -2194,12 +2452,15 @@
         <v>48</v>
       </c>
       <c r="E77" s="2">
-        <v>45002.0</v>
-      </c>
-    </row>
-    <row r="78">
+        <v>45002</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>77.0</v>
+        <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>160</v>
@@ -2211,12 +2472,15 @@
         <v>20</v>
       </c>
       <c r="E78" s="2">
-        <v>45003.0</v>
-      </c>
-    </row>
-    <row r="79">
+        <v>45003</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <v>78.0</v>
+        <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>162</v>
@@ -2228,12 +2492,15 @@
         <v>20</v>
       </c>
       <c r="E79" s="2">
-        <v>45004.0</v>
-      </c>
-    </row>
-    <row r="80">
+        <v>45004</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <v>79.0</v>
+        <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>164</v>
@@ -2245,12 +2512,15 @@
         <v>7</v>
       </c>
       <c r="E80" s="2">
-        <v>45005.0</v>
-      </c>
-    </row>
-    <row r="81">
+        <v>45005</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <v>80.0</v>
+        <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>166</v>
@@ -2262,12 +2532,15 @@
         <v>48</v>
       </c>
       <c r="E81" s="2">
-        <v>45006.0</v>
-      </c>
-    </row>
-    <row r="82">
+        <v>45006</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <v>81.0</v>
+        <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>168</v>
@@ -2279,12 +2552,15 @@
         <v>7</v>
       </c>
       <c r="E82" s="2">
-        <v>45007.0</v>
-      </c>
-    </row>
-    <row r="83">
+        <v>45007</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <v>82.0</v>
+        <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>170</v>
@@ -2296,12 +2572,15 @@
         <v>33</v>
       </c>
       <c r="E83" s="2">
-        <v>45008.0</v>
-      </c>
-    </row>
-    <row r="84">
+        <v>45008</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <v>83.0</v>
+        <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>172</v>
@@ -2313,12 +2592,15 @@
         <v>12</v>
       </c>
       <c r="E84" s="2">
-        <v>45009.0</v>
-      </c>
-    </row>
-    <row r="85">
+        <v>45009</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <v>84.0</v>
+        <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>174</v>
@@ -2330,12 +2612,15 @@
         <v>17</v>
       </c>
       <c r="E85" s="2">
-        <v>45010.0</v>
-      </c>
-    </row>
-    <row r="86">
+        <v>45010</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
-        <v>85.0</v>
+        <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>99</v>
@@ -2347,12 +2632,15 @@
         <v>48</v>
       </c>
       <c r="E86" s="2">
-        <v>45011.0</v>
-      </c>
-    </row>
-    <row r="87">
+        <v>45011</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
-        <v>86.0</v>
+        <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>177</v>
@@ -2364,12 +2652,15 @@
         <v>17</v>
       </c>
       <c r="E87" s="2">
-        <v>45012.0</v>
-      </c>
-    </row>
-    <row r="88">
+        <v>45012</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <v>87.0</v>
+        <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>179</v>
@@ -2381,12 +2672,15 @@
         <v>33</v>
       </c>
       <c r="E88" s="2">
-        <v>45013.0</v>
-      </c>
-    </row>
-    <row r="89">
+        <v>45013</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <v>88.0</v>
+        <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>181</v>
@@ -2398,12 +2692,15 @@
         <v>20</v>
       </c>
       <c r="E89" s="2">
-        <v>45014.0</v>
-      </c>
-    </row>
-    <row r="90">
+        <v>45014</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <v>89.0</v>
+        <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>183</v>
@@ -2415,12 +2712,15 @@
         <v>12</v>
       </c>
       <c r="E90" s="2">
-        <v>45015.0</v>
-      </c>
-    </row>
-    <row r="91">
+        <v>45015</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
-        <v>90.0</v>
+        <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>185</v>
@@ -2432,12 +2732,15 @@
         <v>12</v>
       </c>
       <c r="E91" s="2">
-        <v>45016.0</v>
-      </c>
-    </row>
-    <row r="92">
+        <v>45016</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <v>91.0</v>
+        <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>187</v>
@@ -2449,12 +2752,15 @@
         <v>48</v>
       </c>
       <c r="E92" s="2">
-        <v>45017.0</v>
-      </c>
-    </row>
-    <row r="93">
+        <v>45017</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
-        <v>92.0</v>
+        <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>189</v>
@@ -2466,12 +2772,15 @@
         <v>33</v>
       </c>
       <c r="E93" s="2">
-        <v>45018.0</v>
-      </c>
-    </row>
-    <row r="94">
+        <v>45018</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
-        <v>93.0</v>
+        <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>191</v>
@@ -2483,12 +2792,15 @@
         <v>33</v>
       </c>
       <c r="E94" s="2">
-        <v>45019.0</v>
-      </c>
-    </row>
-    <row r="95">
+        <v>45019</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <v>94.0</v>
+        <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>193</v>
@@ -2500,12 +2812,15 @@
         <v>48</v>
       </c>
       <c r="E95" s="2">
-        <v>45020.0</v>
-      </c>
-    </row>
-    <row r="96">
+        <v>45020</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
-        <v>95.0</v>
+        <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>164</v>
@@ -2517,12 +2832,15 @@
         <v>12</v>
       </c>
       <c r="E96" s="2">
-        <v>45021.0</v>
-      </c>
-    </row>
-    <row r="97">
+        <v>45021</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
-        <v>96.0</v>
+        <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>196</v>
@@ -2534,12 +2852,15 @@
         <v>17</v>
       </c>
       <c r="E97" s="2">
-        <v>45022.0</v>
-      </c>
-    </row>
-    <row r="98">
+        <v>45022</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
-        <v>97.0</v>
+        <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>198</v>
@@ -2551,12 +2872,15 @@
         <v>17</v>
       </c>
       <c r="E98" s="2">
-        <v>45023.0</v>
-      </c>
-    </row>
-    <row r="99">
+        <v>45023</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
-        <v>98.0</v>
+        <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>200</v>
@@ -2568,12 +2892,15 @@
         <v>17</v>
       </c>
       <c r="E99" s="2">
-        <v>45024.0</v>
-      </c>
-    </row>
-    <row r="100">
+        <v>45024</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
-        <v>99.0</v>
+        <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>202</v>
@@ -2585,12 +2912,15 @@
         <v>20</v>
       </c>
       <c r="E100" s="2">
-        <v>45025.0</v>
-      </c>
-    </row>
-    <row r="101">
+        <v>45025</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>204</v>
@@ -2602,10 +2932,13 @@
         <v>17</v>
       </c>
       <c r="E101" s="2">
-        <v>45026.0</v>
+        <v>45026</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>